<commit_message>
Intégration de la solution extension[reason] pour le motif de la demande d'examen c98c647f55473e5f2cd4286d11f173b1edc19084
</commit_message>
<xml_diff>
--- a/imagingServiceRequest/ig/StructureDefinition-fr-service-request-imaging-document.xlsx
+++ b/imagingServiceRequest/ig/StructureDefinition-fr-service-request-imaging-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T08:31:28+00:00</t>
+    <t>2026-08-06T09:04:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -435,9 +435,6 @@
     <t>ServiceRequest.extension</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Extension
 </t>
   </si>
@@ -524,6 +521,9 @@
   </si>
   <si>
     <t>ServiceRequest.extension.extension</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
   <si>
     <t>Extensions are always sliced by (at least) url</t>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
-        <v>135</v>
+        <v>90</v>
       </c>
       <c r="G9" t="s" s="2">
         <v>80</v>
@@ -3213,13 +3213,13 @@
         <v>81</v>
       </c>
       <c r="K9" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L9" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L9" t="s" s="2">
+      <c r="M9" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M9" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -3258,17 +3258,17 @@
         <v>81</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC9" s="2"/>
       <c r="AD9" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE9" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="AF9" t="s" s="2">
         <v>140</v>
-      </c>
-      <c r="AF9" t="s" s="2">
-        <v>141</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>79</v>
@@ -3280,7 +3280,7 @@
         <v>81</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>81</v>
@@ -3300,13 +3300,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>134</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>81</v>
@@ -3328,13 +3328,13 @@
         <v>81</v>
       </c>
       <c r="K10" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="L10" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="L10" t="s" s="2">
+      <c r="M10" t="s" s="2">
         <v>146</v>
-      </c>
-      <c r="M10" t="s" s="2">
-        <v>147</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -3385,7 +3385,7 @@
         <v>81</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>79</v>
@@ -3394,10 +3394,10 @@
         <v>80</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>81</v>
@@ -3417,13 +3417,13 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B11" t="s" s="2">
         <v>134</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D11" t="s" s="2">
         <v>81</v>
@@ -3445,13 +3445,13 @@
         <v>81</v>
       </c>
       <c r="K11" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="L11" t="s" s="2">
         <v>151</v>
       </c>
-      <c r="L11" t="s" s="2">
+      <c r="M11" t="s" s="2">
         <v>152</v>
-      </c>
-      <c r="M11" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -3502,7 +3502,7 @@
         <v>81</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>79</v>
@@ -3511,10 +3511,10 @@
         <v>80</v>
       </c>
       <c r="AI11" t="s" s="2">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK11" t="s" s="2">
         <v>81</v>
@@ -3534,10 +3534,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="B12" t="s" s="2">
         <v>154</v>
-      </c>
-      <c r="B12" t="s" s="2">
-        <v>155</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -3560,13 +3560,13 @@
         <v>81</v>
       </c>
       <c r="K12" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L12" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L12" t="s" s="2">
+      <c r="M12" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M12" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -3617,28 +3617,28 @@
         <v>81</v>
       </c>
       <c r="AF12" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG12" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH12" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI12" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ12" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK12" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL12" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM12" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG12" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH12" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI12" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ12" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK12" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL12" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM12" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN12" t="s" s="2">
         <v>81</v>
@@ -3649,10 +3649,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="B13" t="s" s="2">
         <v>161</v>
-      </c>
-      <c r="B13" t="s" s="2">
-        <v>162</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="G13" t="s" s="2">
         <v>80</v>
@@ -3675,13 +3675,13 @@
         <v>81</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L13" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L13" t="s" s="2">
+      <c r="M13" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M13" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -3720,7 +3720,7 @@
         <v>81</v>
       </c>
       <c r="AB13" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC13" t="s" s="2">
         <v>163</v>
@@ -3729,7 +3729,7 @@
         <v>81</v>
       </c>
       <c r="AE13" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF13" t="s" s="2">
         <v>164</v>
@@ -3744,7 +3744,7 @@
         <v>81</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>81</v>
@@ -3767,7 +3767,7 @@
         <v>165</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C14" t="s" s="2">
         <v>166</v>
@@ -3792,13 +3792,13 @@
         <v>81</v>
       </c>
       <c r="K14" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L14" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L14" t="s" s="2">
+      <c r="M14" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -3861,7 +3861,7 @@
         <v>81</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>81</v>
@@ -3907,13 +3907,13 @@
         <v>81</v>
       </c>
       <c r="K15" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L15" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L15" t="s" s="2">
+      <c r="M15" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M15" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -3964,28 +3964,28 @@
         <v>81</v>
       </c>
       <c r="AF15" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM15" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH15" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN15" t="s" s="2">
         <v>81</v>
@@ -4022,13 +4022,13 @@
         <v>81</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L16" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -4067,7 +4067,7 @@
         <v>81</v>
       </c>
       <c r="AB16" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC16" t="s" s="2">
         <v>163</v>
@@ -4076,7 +4076,7 @@
         <v>81</v>
       </c>
       <c r="AE16" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF16" t="s" s="2">
         <v>164</v>
@@ -4091,7 +4091,7 @@
         <v>81</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK16" t="s" s="2">
         <v>81</v>
@@ -4344,7 +4344,7 @@
         <v>185</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C19" t="s" s="2">
         <v>186</v>
@@ -4369,13 +4369,13 @@
         <v>81</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L19" t="s" s="2">
         <v>187</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -4438,7 +4438,7 @@
         <v>81</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK19" t="s" s="2">
         <v>81</v>
@@ -4484,13 +4484,13 @@
         <v>81</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="M20" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -4541,28 +4541,28 @@
         <v>81</v>
       </c>
       <c r="AF20" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG20" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH20" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI20" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ20" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK20" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL20" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM20" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG20" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH20" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI20" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ20" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK20" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL20" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM20" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN20" t="s" s="2">
         <v>81</v>
@@ -4599,13 +4599,13 @@
         <v>81</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -4644,7 +4644,7 @@
         <v>81</v>
       </c>
       <c r="AB21" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC21" t="s" s="2">
         <v>163</v>
@@ -4653,7 +4653,7 @@
         <v>81</v>
       </c>
       <c r="AE21" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF21" t="s" s="2">
         <v>164</v>
@@ -4668,7 +4668,7 @@
         <v>81</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK21" t="s" s="2">
         <v>81</v>
@@ -4923,7 +4923,7 @@
         <v>193</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C24" t="s" s="2">
         <v>194</v>
@@ -4948,13 +4948,13 @@
         <v>81</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L24" t="s" s="2">
         <v>195</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -5017,7 +5017,7 @@
         <v>81</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK24" t="s" s="2">
         <v>81</v>
@@ -5063,13 +5063,13 @@
         <v>81</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -5120,28 +5120,28 @@
         <v>81</v>
       </c>
       <c r="AF25" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM25" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG25" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH25" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI25" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ25" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK25" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL25" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM25" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN25" t="s" s="2">
         <v>81</v>
@@ -5178,13 +5178,13 @@
         <v>81</v>
       </c>
       <c r="K26" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L26" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L26" t="s" s="2">
+      <c r="M26" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -5223,7 +5223,7 @@
         <v>81</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC26" t="s" s="2">
         <v>163</v>
@@ -5232,7 +5232,7 @@
         <v>81</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF26" t="s" s="2">
         <v>164</v>
@@ -5247,7 +5247,7 @@
         <v>81</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>81</v>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>135</v>
+        <v>90</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>80</v>
@@ -5818,7 +5818,7 @@
         <v>81</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
@@ -5830,7 +5830,7 @@
         <v>81</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>81</v>
@@ -5937,7 +5937,7 @@
         <v>81</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5949,7 +5949,7 @@
         <v>81</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>81</v>
@@ -5972,7 +5972,7 @@
         <v>215</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5995,13 +5995,13 @@
         <v>81</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M33" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -6052,28 +6052,28 @@
         <v>81</v>
       </c>
       <c r="AF33" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL33" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM33" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG33" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH33" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI33" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ33" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK33" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL33" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM33" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>81</v>
@@ -6087,7 +6087,7 @@
         <v>216</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="G34" t="s" s="2">
         <v>80</v>
@@ -6110,13 +6110,13 @@
         <v>81</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L34" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L34" t="s" s="2">
+      <c r="M34" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -6155,7 +6155,7 @@
         <v>81</v>
       </c>
       <c r="AB34" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC34" t="s" s="2">
         <v>163</v>
@@ -6164,7 +6164,7 @@
         <v>81</v>
       </c>
       <c r="AE34" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF34" t="s" s="2">
         <v>164</v>
@@ -6179,7 +6179,7 @@
         <v>81</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>81</v>
@@ -6202,7 +6202,7 @@
         <v>217</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C35" t="s" s="2">
         <v>218</v>
@@ -6227,7 +6227,7 @@
         <v>81</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L35" t="s" s="2">
         <v>219</v>
@@ -6296,7 +6296,7 @@
         <v>81</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>81</v>
@@ -6342,13 +6342,13 @@
         <v>81</v>
       </c>
       <c r="K36" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L36" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L36" t="s" s="2">
+      <c r="M36" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -6399,28 +6399,28 @@
         <v>81</v>
       </c>
       <c r="AF36" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG36" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH36" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI36" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ36" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK36" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL36" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM36" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG36" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH36" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI36" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ36" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK36" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL36" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM36" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>81</v>
@@ -6457,7 +6457,7 @@
         <v>81</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L37" t="s" s="2">
         <v>224</v>
@@ -6504,7 +6504,7 @@
         <v>81</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC37" t="s" s="2">
         <v>163</v>
@@ -6513,7 +6513,7 @@
         <v>81</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF37" t="s" s="2">
         <v>164</v>
@@ -6528,7 +6528,7 @@
         <v>81</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK37" t="s" s="2">
         <v>81</v>
@@ -6537,7 +6537,7 @@
         <v>81</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>81</v>
@@ -6691,7 +6691,7 @@
         <v>81</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L39" t="s" s="2">
         <v>179</v>
@@ -6785,7 +6785,7 @@
         <v>232</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C40" t="s" s="2">
         <v>233</v>
@@ -6810,13 +6810,13 @@
         <v>81</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6879,7 +6879,7 @@
         <v>81</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>81</v>
@@ -6925,13 +6925,13 @@
         <v>81</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6982,28 +6982,28 @@
         <v>81</v>
       </c>
       <c r="AF41" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM41" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG41" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH41" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI41" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ41" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK41" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL41" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM41" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>81</v>
@@ -7040,13 +7040,13 @@
         <v>81</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L42" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L42" t="s" s="2">
+      <c r="M42" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -7085,7 +7085,7 @@
         <v>81</v>
       </c>
       <c r="AB42" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC42" t="s" s="2">
         <v>163</v>
@@ -7094,7 +7094,7 @@
         <v>81</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF42" t="s" s="2">
         <v>164</v>
@@ -7109,7 +7109,7 @@
         <v>81</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>81</v>
@@ -7387,13 +7387,13 @@
         <v>81</v>
       </c>
       <c r="K45" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L45" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L45" t="s" s="2">
+      <c r="M45" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -7444,28 +7444,28 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM45" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG45" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH45" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI45" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ45" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK45" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL45" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM45" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>81</v>
@@ -7502,7 +7502,7 @@
         <v>81</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L46" t="s" s="2">
         <v>224</v>
@@ -7549,7 +7549,7 @@
         <v>81</v>
       </c>
       <c r="AB46" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC46" t="s" s="2">
         <v>163</v>
@@ -7558,7 +7558,7 @@
         <v>81</v>
       </c>
       <c r="AE46" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF46" t="s" s="2">
         <v>164</v>
@@ -7573,7 +7573,7 @@
         <v>81</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK46" t="s" s="2">
         <v>81</v>
@@ -7582,7 +7582,7 @@
         <v>81</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>81</v>
@@ -7738,7 +7738,7 @@
         <v>91</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L48" t="s" s="2">
         <v>257</v>
@@ -7834,7 +7834,7 @@
         <v>264</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C49" t="s" s="2">
         <v>265</v>
@@ -7859,7 +7859,7 @@
         <v>81</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L49" t="s" s="2">
         <v>266</v>
@@ -7932,7 +7932,7 @@
         <v>81</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>81</v>
@@ -7978,13 +7978,13 @@
         <v>81</v>
       </c>
       <c r="K50" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L50" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L50" t="s" s="2">
+      <c r="M50" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -8035,28 +8035,28 @@
         <v>81</v>
       </c>
       <c r="AF50" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM50" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN50" t="s" s="2">
         <v>81</v>
@@ -8093,7 +8093,7 @@
         <v>81</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L51" t="s" s="2">
         <v>224</v>
@@ -8140,7 +8140,7 @@
         <v>81</v>
       </c>
       <c r="AB51" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC51" t="s" s="2">
         <v>163</v>
@@ -8149,7 +8149,7 @@
         <v>81</v>
       </c>
       <c r="AE51" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF51" t="s" s="2">
         <v>164</v>
@@ -8164,7 +8164,7 @@
         <v>81</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>81</v>
@@ -8173,7 +8173,7 @@
         <v>81</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN51" t="s" s="2">
         <v>81</v>
@@ -8661,7 +8661,7 @@
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G56" t="s" s="2">
         <v>90</v>
@@ -8735,7 +8735,7 @@
         <v>81</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -8747,7 +8747,7 @@
         <v>81</v>
       </c>
       <c r="AJ56" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK56" t="s" s="2">
         <v>81</v>
@@ -8770,7 +8770,7 @@
         <v>281</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8793,13 +8793,13 @@
         <v>81</v>
       </c>
       <c r="K57" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L57" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L57" t="s" s="2">
+      <c r="M57" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8850,28 +8850,28 @@
         <v>81</v>
       </c>
       <c r="AF57" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM57" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN57" t="s" s="2">
         <v>81</v>
@@ -8885,7 +8885,7 @@
         <v>282</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8893,7 +8893,7 @@
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="G58" t="s" s="2">
         <v>80</v>
@@ -8908,13 +8908,13 @@
         <v>81</v>
       </c>
       <c r="K58" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L58" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L58" t="s" s="2">
+      <c r="M58" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8953,7 +8953,7 @@
         <v>81</v>
       </c>
       <c r="AB58" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC58" t="s" s="2">
         <v>163</v>
@@ -8962,7 +8962,7 @@
         <v>81</v>
       </c>
       <c r="AE58" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF58" t="s" s="2">
         <v>164</v>
@@ -8977,7 +8977,7 @@
         <v>81</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>81</v>
@@ -9000,7 +9000,7 @@
         <v>283</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C59" t="s" s="2">
         <v>218</v>
@@ -9025,7 +9025,7 @@
         <v>81</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L59" t="s" s="2">
         <v>219</v>
@@ -9094,7 +9094,7 @@
         <v>81</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK59" t="s" s="2">
         <v>81</v>
@@ -9140,13 +9140,13 @@
         <v>81</v>
       </c>
       <c r="K60" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L60" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L60" t="s" s="2">
+      <c r="M60" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
@@ -9197,28 +9197,28 @@
         <v>81</v>
       </c>
       <c r="AF60" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM60" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG60" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH60" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI60" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ60" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK60" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL60" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM60" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN60" t="s" s="2">
         <v>81</v>
@@ -9255,7 +9255,7 @@
         <v>81</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L61" t="s" s="2">
         <v>224</v>
@@ -9302,7 +9302,7 @@
         <v>81</v>
       </c>
       <c r="AB61" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC61" t="s" s="2">
         <v>163</v>
@@ -9311,7 +9311,7 @@
         <v>81</v>
       </c>
       <c r="AE61" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF61" t="s" s="2">
         <v>164</v>
@@ -9326,7 +9326,7 @@
         <v>81</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK61" t="s" s="2">
         <v>81</v>
@@ -9335,7 +9335,7 @@
         <v>81</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN61" t="s" s="2">
         <v>81</v>
@@ -9489,7 +9489,7 @@
         <v>81</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L63" t="s" s="2">
         <v>179</v>
@@ -9583,7 +9583,7 @@
         <v>288</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C64" t="s" s="2">
         <v>233</v>
@@ -9608,13 +9608,13 @@
         <v>81</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M64" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -9677,7 +9677,7 @@
         <v>81</v>
       </c>
       <c r="AJ64" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK64" t="s" s="2">
         <v>81</v>
@@ -9723,13 +9723,13 @@
         <v>81</v>
       </c>
       <c r="K65" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L65" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L65" t="s" s="2">
+      <c r="M65" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M65" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -9780,28 +9780,28 @@
         <v>81</v>
       </c>
       <c r="AF65" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG65" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH65" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM65" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG65" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH65" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI65" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ65" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK65" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL65" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM65" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN65" t="s" s="2">
         <v>81</v>
@@ -9838,13 +9838,13 @@
         <v>81</v>
       </c>
       <c r="K66" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="L66" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="L66" t="s" s="2">
+      <c r="M66" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="M66" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -9883,7 +9883,7 @@
         <v>81</v>
       </c>
       <c r="AB66" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC66" t="s" s="2">
         <v>163</v>
@@ -9892,7 +9892,7 @@
         <v>81</v>
       </c>
       <c r="AE66" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF66" t="s" s="2">
         <v>164</v>
@@ -9907,7 +9907,7 @@
         <v>81</v>
       </c>
       <c r="AJ66" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK66" t="s" s="2">
         <v>81</v>
@@ -10185,13 +10185,13 @@
         <v>81</v>
       </c>
       <c r="K69" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L69" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L69" t="s" s="2">
+      <c r="M69" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -10242,28 +10242,28 @@
         <v>81</v>
       </c>
       <c r="AF69" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG69" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH69" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI69" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ69" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK69" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL69" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM69" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG69" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH69" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI69" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ69" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK69" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL69" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM69" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN69" t="s" s="2">
         <v>81</v>
@@ -10300,7 +10300,7 @@
         <v>81</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L70" t="s" s="2">
         <v>224</v>
@@ -10347,7 +10347,7 @@
         <v>81</v>
       </c>
       <c r="AB70" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC70" t="s" s="2">
         <v>163</v>
@@ -10356,7 +10356,7 @@
         <v>81</v>
       </c>
       <c r="AE70" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF70" t="s" s="2">
         <v>164</v>
@@ -10371,7 +10371,7 @@
         <v>81</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK70" t="s" s="2">
         <v>81</v>
@@ -10380,7 +10380,7 @@
         <v>81</v>
       </c>
       <c r="AM70" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN70" t="s" s="2">
         <v>81</v>
@@ -10536,7 +10536,7 @@
         <v>91</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L72" t="s" s="2">
         <v>257</v>
@@ -10632,7 +10632,7 @@
         <v>298</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C73" t="s" s="2">
         <v>265</v>
@@ -10657,7 +10657,7 @@
         <v>81</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L73" t="s" s="2">
         <v>266</v>
@@ -10730,7 +10730,7 @@
         <v>81</v>
       </c>
       <c r="AJ73" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK73" t="s" s="2">
         <v>81</v>
@@ -10776,13 +10776,13 @@
         <v>81</v>
       </c>
       <c r="K74" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="L74" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="L74" t="s" s="2">
+      <c r="M74" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="M74" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -10833,28 +10833,28 @@
         <v>81</v>
       </c>
       <c r="AF74" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AG74" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH74" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI74" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ74" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK74" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL74" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM74" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="AG74" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH74" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI74" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ74" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK74" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL74" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM74" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="AN74" t="s" s="2">
         <v>81</v>
@@ -10891,7 +10891,7 @@
         <v>81</v>
       </c>
       <c r="K75" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L75" t="s" s="2">
         <v>224</v>
@@ -10938,7 +10938,7 @@
         <v>81</v>
       </c>
       <c r="AB75" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AC75" t="s" s="2">
         <v>163</v>
@@ -10947,7 +10947,7 @@
         <v>81</v>
       </c>
       <c r="AE75" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF75" t="s" s="2">
         <v>164</v>
@@ -10962,7 +10962,7 @@
         <v>81</v>
       </c>
       <c r="AJ75" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK75" t="s" s="2">
         <v>81</v>
@@ -10971,7 +10971,7 @@
         <v>81</v>
       </c>
       <c r="AM75" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AN75" t="s" s="2">
         <v>81</v>
@@ -11472,7 +11472,7 @@
         <v>81</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L80" t="s" s="2">
         <v>306</v>
@@ -11545,7 +11545,7 @@
         <v>81</v>
       </c>
       <c r="AJ80" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AK80" t="s" s="2">
         <v>81</v>
@@ -11645,7 +11645,7 @@
         <v>81</v>
       </c>
       <c r="AE81" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AF81" t="s" s="2">
         <v>310</v>
@@ -15321,7 +15321,7 @@
         <v>91</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L113" t="s" s="2">
         <v>586</v>

</xml_diff>